<commit_message>
Person sheets: public HTML anyone-with-link view
</commit_message>
<xml_diff>
--- a/Recovery-Desk.xlsx
+++ b/Recovery-Desk.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Added red" sheetId="7" r:id="rId7"/>
     <sheet name="Reduced green" sheetId="8" r:id="rId8"/>
     <sheet name="All overdue" sheetId="9" r:id="rId9"/>
-    <sheet name="Control" sheetId="10" r:id="rId10"/>
+    <sheet name="NACH not live" sheetId="10" r:id="rId10"/>
   </sheets>
 </workbook>
 </file>
@@ -406,24 +406,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:E12"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Perfect Finmart Recovery Desk — public sheet</v>
+        <v>Recovery Desk</v>
+      </c>
+      <c r="B1" t="str">
+        <v>2026-09-19</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Dump 2026-09-19 vs start 2026-09-16</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
+        <v>Headline</v>
+      </c>
+      <c r="B2" t="str">
         <v>19 Sep is mixed vs 16 Sep.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Vs 16 Sep</v>
       </c>
     </row>
     <row r="5">
@@ -431,18 +438,21 @@
         <v>What</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-09-16</v>
+        <v>16 Sep</v>
       </c>
       <c r="C5" t="str">
-        <v>2026-09-19</v>
+        <v>This mail</v>
       </c>
       <c r="D5" t="str">
-        <v>Change</v>
+        <v>Delta cases</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Delta ₹</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Cases not paid</v>
+        <v>Unpaid cases</v>
       </c>
       <c r="B6">
         <v>598</v>
@@ -452,6 +462,9 @@
       </c>
       <c r="D6">
         <v>-173</v>
+      </c>
+      <c r="E6" t="str">
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -464,209 +477,147 @@
       <c r="C7">
         <v>22313607</v>
       </c>
-      <c r="D7">
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7">
         <v>-3021599</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Late 91 days+</v>
+        <v>1 EMI overdue</v>
       </c>
       <c r="B8">
-        <v>190</v>
+        <v>279</v>
       </c>
       <c r="C8">
-        <v>206</v>
+        <v>131</v>
       </c>
       <c r="D8">
-        <v>16</v>
+        <v>-148</v>
+      </c>
+      <c r="E8">
+        <v>-2052688</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>More than 1, less than 2</v>
+      </c>
+      <c r="B9">
+        <v>69</v>
+      </c>
+      <c r="C9">
+        <v>42</v>
+      </c>
+      <c r="D9">
+        <v>-27</v>
+      </c>
+      <c r="E9">
+        <v>-716354</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Desk</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Person</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Cases today</v>
-      </c>
-      <c r="D10" t="str">
-        <v>Cases 16 Sep</v>
-      </c>
-      <c r="E10" t="str">
-        <v>Δ cases</v>
-      </c>
-      <c r="F10" t="str">
-        <v>Overdue ₹ today</v>
-      </c>
-      <c r="G10" t="str">
-        <v>Overdue ₹ 16 Sep</v>
-      </c>
-      <c r="H10" t="str">
-        <v>Δ ₹</v>
+        <v>2 to less than 3</v>
+      </c>
+      <c r="B10">
+        <v>60</v>
+      </c>
+      <c r="C10">
+        <v>46</v>
+      </c>
+      <c r="D10">
+        <v>-14</v>
+      </c>
+      <c r="E10">
+        <v>-612333</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>1 EMI overdue</v>
+        <v>3 to 6 months</v>
       </c>
       <c r="B11">
-        <v>1</v>
+        <v>95</v>
       </c>
       <c r="C11">
-        <v>131</v>
+        <v>103</v>
       </c>
       <c r="D11">
-        <v>279</v>
+        <v>8</v>
       </c>
       <c r="E11">
-        <v>-148</v>
-      </c>
-      <c r="F11">
-        <v>1740256</v>
-      </c>
-      <c r="G11">
-        <v>3792944</v>
-      </c>
-      <c r="H11">
-        <v>-2052688</v>
+        <v>-251277</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>More than 1, less than 2</v>
+        <v>More than 6 months</v>
       </c>
       <c r="B12">
-        <v>2</v>
+        <v>95</v>
       </c>
       <c r="C12">
-        <v>42</v>
+        <v>103</v>
       </c>
       <c r="D12">
-        <v>69</v>
+        <v>8</v>
       </c>
       <c r="E12">
-        <v>-27</v>
-      </c>
-      <c r="F12">
-        <v>962356</v>
-      </c>
-      <c r="G12">
-        <v>1678710</v>
-      </c>
-      <c r="H12">
-        <v>-716354</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>2 to less than 3</v>
-      </c>
-      <c r="B13">
-        <v>3</v>
-      </c>
-      <c r="C13">
-        <v>46</v>
-      </c>
-      <c r="D13">
-        <v>60</v>
-      </c>
-      <c r="E13">
-        <v>-14</v>
-      </c>
-      <c r="F13">
-        <v>1709022</v>
-      </c>
-      <c r="G13">
-        <v>2321355</v>
-      </c>
-      <c r="H13">
-        <v>-612333</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>3 to 6 months</v>
-      </c>
-      <c r="B14">
-        <v>4</v>
-      </c>
-      <c r="C14">
-        <v>103</v>
-      </c>
-      <c r="D14">
-        <v>95</v>
-      </c>
-      <c r="E14">
-        <v>8</v>
-      </c>
-      <c r="F14">
-        <v>5659761</v>
-      </c>
-      <c r="G14">
-        <v>5911038</v>
-      </c>
-      <c r="H14">
-        <v>-251277</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>More than 6 months</v>
-      </c>
-      <c r="B15">
-        <v>5</v>
-      </c>
-      <c r="C15">
-        <v>103</v>
-      </c>
-      <c r="D15">
-        <v>95</v>
-      </c>
-      <c r="E15">
-        <v>8</v>
-      </c>
-      <c r="F15">
-        <v>12242212</v>
-      </c>
-      <c r="G15">
-        <v>11631159</v>
-      </c>
-      <c r="H15">
         <v>611053</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E12"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:I45"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="28.83203125" customWidth="1"/>
     <col min="3" max="3" width="12.83203125" customWidth="1"/>
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Person</v>
+        <v>S.no</v>
       </c>
       <c r="B1" t="str">
+        <v>File / case no.</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Name</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Days late</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Overdue ₹</v>
+      </c>
+      <c r="F1" t="str">
+        <v>EMI ₹</v>
+      </c>
+      <c r="G1" t="str">
+        <v>PDC</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Mobile</v>
+      </c>
+      <c r="I1" t="str">
         <v>Desk</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Cases</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Overdue ₹</v>
       </c>
     </row>
     <row r="2">
@@ -674,13 +625,28 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>1 EMI overdue</v>
-      </c>
-      <c r="C2">
-        <v>131</v>
+        <v>FD460083</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Munna Kumar S/O Vijay  Singh</v>
       </c>
       <c r="D2">
-        <v>1740256</v>
+        <v>94</v>
+      </c>
+      <c r="E2">
+        <v>281013</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2" t="str">
+        <v>PDC</v>
+      </c>
+      <c r="H2" t="str">
+        <v>9717920033</v>
+      </c>
+      <c r="I2" t="str">
+        <v>3–6 m</v>
       </c>
     </row>
     <row r="3">
@@ -688,13 +654,28 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>More than 1, less than 2</v>
-      </c>
-      <c r="C3">
-        <v>42</v>
+        <v>FS460049</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Arvind Kumar Dhawan S/O Mani Ram Dhawan</v>
       </c>
       <c r="D3">
-        <v>962356</v>
+        <v>71</v>
+      </c>
+      <c r="E3">
+        <v>141429</v>
+      </c>
+      <c r="F3">
+        <v>47143</v>
+      </c>
+      <c r="G3" t="str">
+        <v>NPDC</v>
+      </c>
+      <c r="H3" t="str">
+        <v>9718572702</v>
+      </c>
+      <c r="I3" t="str">
+        <v>2–3 m</v>
       </c>
     </row>
     <row r="4">
@@ -702,13 +683,28 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>2 to less than 3</v>
-      </c>
-      <c r="C4">
-        <v>46</v>
+        <v>FP440417</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Mohammad Munna Khan S/O Kafil  Khan</v>
       </c>
       <c r="D4">
-        <v>1709022</v>
+        <v>178</v>
+      </c>
+      <c r="E4">
+        <v>111048</v>
+      </c>
+      <c r="F4">
+        <v>18536</v>
+      </c>
+      <c r="G4" t="str">
+        <v>NPDC</v>
+      </c>
+      <c r="H4" t="str">
+        <v>9650402942</v>
+      </c>
+      <c r="I4" t="str">
+        <v>3–6 m</v>
       </c>
     </row>
     <row r="5">
@@ -716,13 +712,28 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>3 to 6 months</v>
-      </c>
-      <c r="C5">
-        <v>103</v>
+        <v>FP450573</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Vikas . S/O Roshan  Lal</v>
       </c>
       <c r="D5">
-        <v>5659761</v>
+        <v>86</v>
+      </c>
+      <c r="E5">
+        <v>84951</v>
+      </c>
+      <c r="F5">
+        <v>28317</v>
+      </c>
+      <c r="G5" t="str">
+        <v>NPDC</v>
+      </c>
+      <c r="H5" t="str">
+        <v>7683059184</v>
+      </c>
+      <c r="I5" t="str">
+        <v>2–3 m</v>
       </c>
     </row>
     <row r="6">
@@ -730,18 +741,1164 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>More than 6 months</v>
-      </c>
-      <c r="C6">
-        <v>103</v>
+        <v>FP440567</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Poonam Devi C/O Ramesh  Chand</v>
       </c>
       <c r="D6">
-        <v>12242212</v>
+        <v>122</v>
+      </c>
+      <c r="E6">
+        <v>54672</v>
+      </c>
+      <c r="F6">
+        <v>16667</v>
+      </c>
+      <c r="G6" t="str">
+        <v>PDC</v>
+      </c>
+      <c r="H6" t="str">
+        <v>9811021922</v>
+      </c>
+      <c r="I6" t="str">
+        <v>3–6 m</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>FS450656</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Roshani Devi W/O Gopal Prasad Chaurasiya</v>
+      </c>
+      <c r="D7">
+        <v>86</v>
+      </c>
+      <c r="E7">
+        <v>45501</v>
+      </c>
+      <c r="F7">
+        <v>15167</v>
+      </c>
+      <c r="G7" t="str">
+        <v>NPDC</v>
+      </c>
+      <c r="H7" t="str">
+        <v>7065396166</v>
+      </c>
+      <c r="I7" t="str">
+        <v>2–3 m</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="str">
+        <v>FS450548</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Kaleecharan . S/O Hari  Ram</v>
+      </c>
+      <c r="D8">
+        <v>132</v>
+      </c>
+      <c r="E8">
+        <v>41115</v>
+      </c>
+      <c r="F8">
+        <v>8223</v>
+      </c>
+      <c r="G8" t="str">
+        <v>NPDC</v>
+      </c>
+      <c r="H8" t="str">
+        <v>8765148147</v>
+      </c>
+      <c r="I8" t="str">
+        <v>3–6 m</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="str">
+        <v>FP450102</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Shobha Devi W/O Jagdish  Ram</v>
+      </c>
+      <c r="D9">
+        <v>91</v>
+      </c>
+      <c r="E9">
+        <v>39999</v>
+      </c>
+      <c r="F9">
+        <v>13333</v>
+      </c>
+      <c r="G9" t="str">
+        <v>NPDC</v>
+      </c>
+      <c r="H9" t="str">
+        <v>7982892737</v>
+      </c>
+      <c r="I9" t="str">
+        <v>3–6 m</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="str">
+        <v>FP450039</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Gopal Singh Bisht S/O Govind Singh Bisht</v>
+      </c>
+      <c r="D10">
+        <v>25</v>
+      </c>
+      <c r="E10">
+        <v>19723</v>
+      </c>
+      <c r="F10">
+        <v>19723</v>
+      </c>
+      <c r="G10" t="str">
+        <v>NPDC</v>
+      </c>
+      <c r="H10" t="str">
+        <v>9999944493</v>
+      </c>
+      <c r="I10" t="str">
+        <v>1 EMI</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>FP450334</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Mohd Mozahid S/O Mohd Yusuf Ali</v>
+      </c>
+      <c r="D11">
+        <v>40</v>
+      </c>
+      <c r="E11">
+        <v>16320</v>
+      </c>
+      <c r="F11">
+        <v>12657</v>
+      </c>
+      <c r="G11" t="str">
+        <v>NPDC</v>
+      </c>
+      <c r="H11" t="str">
+        <v>9958256651</v>
+      </c>
+      <c r="I11" t="str">
+        <v>1–2 m</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>FP460157</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Ranju Devi W/O Prem  Lal</v>
+      </c>
+      <c r="D12">
+        <v>4</v>
+      </c>
+      <c r="E12">
+        <v>16042</v>
+      </c>
+      <c r="F12">
+        <v>16042</v>
+      </c>
+      <c r="G12" t="str">
+        <v>NPDC</v>
+      </c>
+      <c r="H12" t="str">
+        <v>8651426623</v>
+      </c>
+      <c r="I12" t="str">
+        <v>1 EMI</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>FS460169</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Suman . W/O Manoj  Kumar</v>
+      </c>
+      <c r="D13">
+        <v>4</v>
+      </c>
+      <c r="E13">
+        <v>15500</v>
+      </c>
+      <c r="F13">
+        <v>15500</v>
+      </c>
+      <c r="G13" t="str">
+        <v>NPDC</v>
+      </c>
+      <c r="H13" t="str">
+        <v>8882337869</v>
+      </c>
+      <c r="I13" t="str">
+        <v>1 EMI</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>FP450502</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Reema . W/O Pankaj  .</v>
+      </c>
+      <c r="D14">
+        <v>4</v>
+      </c>
+      <c r="E14">
+        <v>12083</v>
+      </c>
+      <c r="F14">
+        <v>12083</v>
+      </c>
+      <c r="G14" t="str">
+        <v>PDC</v>
+      </c>
+      <c r="H14" t="str">
+        <v>8810535551</v>
+      </c>
+      <c r="I14" t="str">
+        <v>1 EMI</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>FP450596</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Noorjhan Khatoon W/O Md  Sanaullah</v>
+      </c>
+      <c r="D15">
+        <v>4</v>
+      </c>
+      <c r="E15">
+        <v>11994</v>
+      </c>
+      <c r="F15">
+        <v>11994</v>
+      </c>
+      <c r="G15" t="str">
+        <v>PDC</v>
+      </c>
+      <c r="H15" t="str">
+        <v>8587038949</v>
+      </c>
+      <c r="I15" t="str">
+        <v>1 EMI</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>FU450579</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Sonu Kumar Kamat S/O Lalbabu  Kamat</v>
+      </c>
+      <c r="D16">
+        <v>25</v>
+      </c>
+      <c r="E16">
+        <v>4500</v>
+      </c>
+      <c r="F16">
+        <v>4500</v>
+      </c>
+      <c r="G16" t="str">
+        <v>NPDC</v>
+      </c>
+      <c r="H16" t="str">
+        <v>9304848103</v>
+      </c>
+      <c r="I16" t="str">
+        <v>1 EMI</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="str">
+        <v>FU460183</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Awadhesh . S/O Ramchandra  Singh</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17">
+        <v>0</v>
+      </c>
+      <c r="F17">
+        <v>0</v>
+      </c>
+      <c r="G17" t="str">
+        <v>NPDC</v>
+      </c>
+      <c r="H17" t="str">
+        <v>7011694664</v>
+      </c>
+      <c r="I17" t="str">
+        <v>current</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="str">
+        <v>FP440557</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Babita Devi W/O Dhurender  Shani</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18">
+        <v>0</v>
+      </c>
+      <c r="F18">
+        <v>10208</v>
+      </c>
+      <c r="G18" t="str">
+        <v>PDC</v>
+      </c>
+      <c r="H18" t="str">
+        <v>8800904341</v>
+      </c>
+      <c r="I18" t="str">
+        <v>current</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="str">
+        <v>FP460194</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Chote Lal S/O Jogindar  Yadav</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <v>0</v>
+      </c>
+      <c r="F19">
+        <v>0</v>
+      </c>
+      <c r="G19" t="str">
+        <v>NPDC</v>
+      </c>
+      <c r="H19" t="str">
+        <v>9319769219</v>
+      </c>
+      <c r="I19" t="str">
+        <v>current</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="str">
+        <v>FS460179</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Chunnu Prasad Prajapati S/O Bandi Prasad Prajapati</v>
+      </c>
+      <c r="D20">
+        <v>0</v>
+      </c>
+      <c r="E20">
+        <v>0</v>
+      </c>
+      <c r="F20">
+        <v>0</v>
+      </c>
+      <c r="G20" t="str">
+        <v>NPDC</v>
+      </c>
+      <c r="H20" t="str">
+        <v>9899044327</v>
+      </c>
+      <c r="I20" t="str">
+        <v>current</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="str">
+        <v>FP460142</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Geeta Devi W/O Sujeet  Chaudhari</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21">
+        <v>0</v>
+      </c>
+      <c r="F21">
+        <v>0</v>
+      </c>
+      <c r="G21" t="str">
+        <v>NPDC</v>
+      </c>
+      <c r="H21" t="str">
+        <v>8287094872</v>
+      </c>
+      <c r="I21" t="str">
+        <v>current</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="str">
+        <v>FP450211</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Indrawati . S/O Subay  Singh</v>
+      </c>
+      <c r="D22">
+        <v>0</v>
+      </c>
+      <c r="E22">
+        <v>0</v>
+      </c>
+      <c r="F22">
+        <v>11161</v>
+      </c>
+      <c r="G22" t="str">
+        <v>PDC</v>
+      </c>
+      <c r="H22" t="str">
+        <v>9968917511</v>
+      </c>
+      <c r="I22" t="str">
+        <v>current</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="str">
+        <v>FP460172</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Lalit Mohan S/O Bishan  Singh</v>
+      </c>
+      <c r="D23">
+        <v>0</v>
+      </c>
+      <c r="E23">
+        <v>0</v>
+      </c>
+      <c r="F23">
+        <v>0</v>
+      </c>
+      <c r="G23" t="str">
+        <v>NPDC</v>
+      </c>
+      <c r="H23" t="str">
+        <v>9540788199</v>
+      </c>
+      <c r="I23" t="str">
+        <v>current</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="str">
+        <v>FS460193</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Pinku Devi W/O Govind  Ram</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24">
+        <v>0</v>
+      </c>
+      <c r="F24">
+        <v>0</v>
+      </c>
+      <c r="G24" t="str">
+        <v>NPDC</v>
+      </c>
+      <c r="H24" t="str">
+        <v>7827653484</v>
+      </c>
+      <c r="I24" t="str">
+        <v>current</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="str">
+        <v>FP450342</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Poonam Pandey S/O Badri Prasad Mishar</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25">
+        <v>0</v>
+      </c>
+      <c r="F25">
+        <v>18728</v>
+      </c>
+      <c r="G25" t="str">
+        <v>PDC</v>
+      </c>
+      <c r="H25" t="str">
+        <v>9289055699</v>
+      </c>
+      <c r="I25" t="str">
+        <v>current</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="str">
+        <v>FP460039</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Veena Rajput W/O Sanjay  .</v>
+      </c>
+      <c r="D26">
+        <v>0</v>
+      </c>
+      <c r="E26">
+        <v>0</v>
+      </c>
+      <c r="F26">
+        <v>8750</v>
+      </c>
+      <c r="G26" t="str">
+        <v>NPDC</v>
+      </c>
+      <c r="H26" t="str">
+        <v>8750977089</v>
+      </c>
+      <c r="I26" t="str">
+        <v>current</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="str">
+        <v>FS460181</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Phool Kumari W/O Jagdish Prasad Yadav</v>
+      </c>
+      <c r="D27">
+        <v>0</v>
+      </c>
+      <c r="E27">
+        <v>0</v>
+      </c>
+      <c r="F27">
+        <v>0</v>
+      </c>
+      <c r="G27" t="str">
+        <v>NPDC</v>
+      </c>
+      <c r="H27" t="str">
+        <v>9310735020</v>
+      </c>
+      <c r="I27" t="str">
+        <v>current</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="str">
+        <v>FS460184</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Pooja Devi W/O Videsh Kumar Pal</v>
+      </c>
+      <c r="D28">
+        <v>0</v>
+      </c>
+      <c r="E28">
+        <v>0</v>
+      </c>
+      <c r="F28">
+        <v>0</v>
+      </c>
+      <c r="G28" t="str">
+        <v>NPDC</v>
+      </c>
+      <c r="H28" t="str">
+        <v>9540350901</v>
+      </c>
+      <c r="I28" t="str">
+        <v>current</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="str">
+        <v>FP450472</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Kishan . S/O Shahab  Singh</v>
+      </c>
+      <c r="D29">
+        <v>0</v>
+      </c>
+      <c r="E29">
+        <v>0</v>
+      </c>
+      <c r="F29">
+        <v>13533</v>
+      </c>
+      <c r="G29" t="str">
+        <v>NPDC</v>
+      </c>
+      <c r="H29" t="str">
+        <v>9310257076</v>
+      </c>
+      <c r="I29" t="str">
+        <v>current</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="str">
+        <v>FP450609</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Maheshwari Devi W/O Omveer  Singh</v>
+      </c>
+      <c r="D30">
+        <v>0</v>
+      </c>
+      <c r="E30">
+        <v>0</v>
+      </c>
+      <c r="F30">
+        <v>20000</v>
+      </c>
+      <c r="G30" t="str">
+        <v>PDC</v>
+      </c>
+      <c r="H30" t="str">
+        <v>8076404199</v>
+      </c>
+      <c r="I30" t="str">
+        <v>current</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="str">
+        <v>FP450470</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Suresh Kumar Yadav S/O Jagveer  Yadav</v>
+      </c>
+      <c r="D31">
+        <v>0</v>
+      </c>
+      <c r="E31">
+        <v>0</v>
+      </c>
+      <c r="F31">
+        <v>6000</v>
+      </c>
+      <c r="G31" t="str">
+        <v>NPDC</v>
+      </c>
+      <c r="H31" t="str">
+        <v>9818847320</v>
+      </c>
+      <c r="I31" t="str">
+        <v>current</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="str">
+        <v>FP460176</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Taniya . D/O Sandeep  .</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32">
+        <v>0</v>
+      </c>
+      <c r="F32">
+        <v>0</v>
+      </c>
+      <c r="G32" t="str">
+        <v>NPDC</v>
+      </c>
+      <c r="H32" t="str">
+        <v>7217602260</v>
+      </c>
+      <c r="I32" t="str">
+        <v>current</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="str">
+        <v>FP450294</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Topona Rani Ray W/O Uttam Kumar Ray</v>
+      </c>
+      <c r="D33">
+        <v>0</v>
+      </c>
+      <c r="E33">
+        <v>0</v>
+      </c>
+      <c r="F33">
+        <v>12400</v>
+      </c>
+      <c r="G33" t="str">
+        <v>NPDC</v>
+      </c>
+      <c r="H33" t="str">
+        <v>7042149901</v>
+      </c>
+      <c r="I33" t="str">
+        <v>current</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="str">
+        <v>FP431256</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Manish Moudgill S/O Jeevan Lal Moudgill</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+      <c r="E34">
+        <v>0</v>
+      </c>
+      <c r="F34">
+        <v>0</v>
+      </c>
+      <c r="G34" t="str">
+        <v>PDC</v>
+      </c>
+      <c r="H34" t="str">
+        <v>9811036072</v>
+      </c>
+      <c r="I34" t="str">
+        <v>current</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="str">
+        <v>FP440569</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Minesh . W/O Prahalad  .</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35">
+        <v>0</v>
+      </c>
+      <c r="F35">
+        <v>6400</v>
+      </c>
+      <c r="G35" t="str">
+        <v>NPDC</v>
+      </c>
+      <c r="H35" t="str">
+        <v>9761276759</v>
+      </c>
+      <c r="I35" t="str">
+        <v>current</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" t="str">
+        <v>FP440103</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Bhagwan Dass Chaudhary S/O Upinder  Chaudhary</v>
+      </c>
+      <c r="D36">
+        <v>0</v>
+      </c>
+      <c r="E36">
+        <v>0</v>
+      </c>
+      <c r="F36">
+        <v>21654</v>
+      </c>
+      <c r="G36" t="str">
+        <v>PDC</v>
+      </c>
+      <c r="H36" t="str">
+        <v>9818374631</v>
+      </c>
+      <c r="I36" t="str">
+        <v>current</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" t="str">
+        <v>FP440016</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Anil Yadav S/O Naresh  Yadav</v>
+      </c>
+      <c r="D37">
+        <v>0</v>
+      </c>
+      <c r="E37">
+        <v>0</v>
+      </c>
+      <c r="F37">
+        <v>12889</v>
+      </c>
+      <c r="G37" t="str">
+        <v>PDC</v>
+      </c>
+      <c r="H37" t="str">
+        <v>9891569267</v>
+      </c>
+      <c r="I37" t="str">
+        <v>current</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" t="str">
+        <v>FP450562</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Anju Devi W/O Raghunandan  Ram</v>
+      </c>
+      <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38">
+        <v>0</v>
+      </c>
+      <c r="F38">
+        <v>10208</v>
+      </c>
+      <c r="G38" t="str">
+        <v>NPDC</v>
+      </c>
+      <c r="H38" t="str">
+        <v>8130758076</v>
+      </c>
+      <c r="I38" t="str">
+        <v>current</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39" t="str">
+        <v>FP450479</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Arvind . S/O Kripa Shankar Gupta</v>
+      </c>
+      <c r="D39">
+        <v>0</v>
+      </c>
+      <c r="E39">
+        <v>0</v>
+      </c>
+      <c r="F39">
+        <v>15333</v>
+      </c>
+      <c r="G39" t="str">
+        <v>PDC</v>
+      </c>
+      <c r="H39" t="str">
+        <v>9911980079</v>
+      </c>
+      <c r="I39" t="str">
+        <v>current</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40" t="str">
+        <v>FP460197</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Dinesh Sah S/O Ramautar  Sah</v>
+      </c>
+      <c r="D40">
+        <v>0</v>
+      </c>
+      <c r="E40">
+        <v>0</v>
+      </c>
+      <c r="F40">
+        <v>0</v>
+      </c>
+      <c r="G40" t="str">
+        <v>NPDC</v>
+      </c>
+      <c r="H40" t="str">
+        <v>7827776285</v>
+      </c>
+      <c r="I40" t="str">
+        <v>current</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41" t="str">
+        <v>FP460178</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Pushpa Devi W/O Deevan  .</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41">
+        <v>0</v>
+      </c>
+      <c r="F41">
+        <v>0</v>
+      </c>
+      <c r="G41" t="str">
+        <v>NPDC</v>
+      </c>
+      <c r="H41" t="str">
+        <v>9716531871</v>
+      </c>
+      <c r="I41" t="str">
+        <v>current</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42" t="str">
+        <v>FP450047</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Rakesh Kumar S/O Todiram  .</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+      <c r="E42">
+        <v>0</v>
+      </c>
+      <c r="F42">
+        <v>11833</v>
+      </c>
+      <c r="G42" t="str">
+        <v>PDC</v>
+      </c>
+      <c r="H42" t="str">
+        <v>8826266520</v>
+      </c>
+      <c r="I42" t="str">
+        <v>current</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43" t="str">
+        <v>FS450576</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Sunita Rani W/O Vashist  Jha</v>
+      </c>
+      <c r="D43">
+        <v>0</v>
+      </c>
+      <c r="E43">
+        <v>0</v>
+      </c>
+      <c r="F43">
+        <v>12984</v>
+      </c>
+      <c r="G43" t="str">
+        <v>PDC</v>
+      </c>
+      <c r="H43" t="str">
+        <v>9718671982</v>
+      </c>
+      <c r="I43" t="str">
+        <v>current</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44" t="str">
+        <v>FP440540</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Mamta Mishra W/O Mukesh Kumar Mishra</v>
+      </c>
+      <c r="D44">
+        <v>0</v>
+      </c>
+      <c r="E44">
+        <v>-3</v>
+      </c>
+      <c r="F44">
+        <v>5208</v>
+      </c>
+      <c r="G44" t="str">
+        <v>PDC</v>
+      </c>
+      <c r="H44" t="str">
+        <v>9718469121</v>
+      </c>
+      <c r="I44" t="str">
+        <v>current</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45" t="str">
+        <v>FP450089</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Rohit Singh S/O Surender Pal Singh</v>
+      </c>
+      <c r="D45">
+        <v>0</v>
+      </c>
+      <c r="E45">
+        <v>-6120</v>
+      </c>
+      <c r="F45">
+        <v>31223</v>
+      </c>
+      <c r="G45" t="str">
+        <v>NPDC</v>
+      </c>
+      <c r="H45" t="str">
+        <v>8800178488</v>
+      </c>
+      <c r="I45" t="str">
+        <v>current</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I45"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>